<commit_message>
feat(skill): replace physics queries with entity body checks
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/UnitConfig.xlsx
+++ b/Design/Excel/ET/Datas/Game/UnitConfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ugit\myGameDevelopmentKit\Design\Excel\ET\Datas\Game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ADDB496-F0B6-474A-A039-B18CB36C7E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17839334-0EDE-44A8-9B08-959B9AC9A79D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
   <si>
     <t>##var</t>
   </si>
@@ -61,12 +61,6 @@
     <t>string</t>
   </si>
   <si>
-    <t>int&amp;group=c</t>
-  </si>
-  <si>
-    <t>int&amp;group=s</t>
-  </si>
-  <si>
     <t>测试说明</t>
   </si>
   <si>
@@ -98,6 +92,26 @@
   </si>
   <si>
     <t>带有强力攻击技能2</t>
+  </si>
+  <si>
+    <t>Width</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>宽度</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shape</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>形状</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -495,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.08984375" style="2" customWidth="1"/>
@@ -503,14 +517,17 @@
     <col min="4" max="5" width="12.6328125" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.08984375" style="2" customWidth="1"/>
     <col min="7" max="7" width="9.6328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="28.7265625" style="2" customWidth="1"/>
-    <col min="9" max="10" width="11.7265625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="6.7265625" style="2" customWidth="1"/>
-    <col min="12" max="12" width="9" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="9" style="2"/>
+    <col min="8" max="8" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" style="2" customWidth="1"/>
+    <col min="10" max="10" width="6.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.7265625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="9" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -534,13 +551,19 @@
         <v>9</v>
       </c>
       <c r="I1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -564,13 +587,19 @@
         <v>2</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>14</v>
+        <v>27</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -582,25 +611,31 @@
         <v>6</v>
       </c>
       <c r="E3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="I3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>20</v>
-      </c>
     </row>
-    <row r="4" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="1">
         <v>1001</v>
@@ -612,25 +647,31 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
       </c>
       <c r="I4" s="1">
-        <v>178</v>
+        <v>1</v>
       </c>
       <c r="J4" s="1">
+        <v>2</v>
+      </c>
+      <c r="K4" s="1">
+        <v>4</v>
+      </c>
+      <c r="L4" s="1">
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="1">
         <v>2001</v>
@@ -642,21 +683,27 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="H5" s="1">
         <v>2</v>
       </c>
       <c r="I5" s="1">
-        <v>278</v>
+        <v>1</v>
       </c>
       <c r="J5" s="1">
+        <v>2</v>
+      </c>
+      <c r="K5" s="1">
+        <v>4</v>
+      </c>
+      <c r="L5" s="1">
         <v>78</v>
       </c>
     </row>

</xml_diff>